<commit_message>
Building out the pipeline - almost to the Hello Device
</commit_message>
<xml_diff>
--- a/Design/Workflow Sketch.xlsx
+++ b/Design/Workflow Sketch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llmdevice\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21A3B6C-0F74-449F-A034-EB130C2CF277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3997F65-22C6-4B65-8A40-E4B351816EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -204,15 +204,9 @@
     <t>Check for Drivers</t>
   </si>
   <si>
-    <t>Install Drivers</t>
-  </si>
-  <si>
     <t>Confirm the type of system we are working on through Linux commands. Then, using only official sources, see if we need drivers for our system</t>
   </si>
   <si>
-    <t>Install any necessary device drivers</t>
-  </si>
-  <si>
     <t>Check if we will need certain device drivers to implement our goals</t>
   </si>
   <si>
@@ -228,9 +222,6 @@
     <t>Text, Linux Shell Access</t>
   </si>
   <si>
-    <t>Agentically assist the user through downloading and installing the necessary drivers for the device, so device is recognized on the computer.</t>
-  </si>
-  <si>
     <t>Justification for why it thinks the connection was successful</t>
   </si>
   <si>
@@ -430,6 +421,15 @@
   </si>
   <si>
     <t>HUMAN VETS ALL OF LEVEL 3 (manually inspecting the data outputs, and/or trying out simple experiment orchestration runs)</t>
+  </si>
+  <si>
+    <t>Install Drivers and Core Libraries</t>
+  </si>
+  <si>
+    <t>Install any necessary device drivers and low-level libraries for Python</t>
+  </si>
+  <si>
+    <t>Agentically assist the user through downloading and installing the necessary drivers for the device, so device is recognized on the computer. You also need any core, low-level Python libraries that would make basic hello, world type communication work.</t>
   </si>
 </sst>
 </file>
@@ -957,7 +957,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
         <v>49</v>
@@ -989,7 +989,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
@@ -1013,329 +1013,329 @@
         <v>14</v>
       </c>
       <c r="I8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H9" t="s">
         <v>14</v>
       </c>
       <c r="I9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" t="s">
+        <v>134</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" t="s">
         <v>67</v>
-      </c>
-      <c r="H11" t="s">
-        <v>65</v>
-      </c>
-      <c r="I11" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
         <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" t="s">
         <v>64</v>
       </c>
-      <c r="F12" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" t="s">
-        <v>66</v>
-      </c>
       <c r="J12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
       <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" t="s">
         <v>79</v>
       </c>
-      <c r="G13" t="s">
-        <v>98</v>
-      </c>
-      <c r="H13" t="s">
-        <v>82</v>
-      </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J13" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
         <v>99</v>
       </c>
-      <c r="D14" t="s">
-        <v>91</v>
-      </c>
-      <c r="E14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I14" t="s">
+        <v>90</v>
+      </c>
+      <c r="J14" t="s">
         <v>93</v>
-      </c>
-      <c r="J14" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
         <v>86</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>97</v>
+      </c>
+      <c r="D15" t="s">
         <v>89</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
         <v>100</v>
       </c>
-      <c r="D15" t="s">
-        <v>92</v>
-      </c>
-      <c r="E15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" t="s">
-        <v>103</v>
-      </c>
       <c r="H15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" t="s">
+        <v>111</v>
+      </c>
+      <c r="E17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" t="s">
         <v>113</v>
       </c>
-      <c r="B17" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" t="s">
-        <v>114</v>
-      </c>
-      <c r="E17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" t="s">
-        <v>116</v>
-      </c>
       <c r="I17" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
+        <v>101</v>
+      </c>
+      <c r="E18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" t="s">
+        <v>87</v>
+      </c>
+      <c r="I18" t="s">
         <v>104</v>
-      </c>
-      <c r="E18" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" t="s">
-        <v>90</v>
-      </c>
-      <c r="I18" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>107</v>
+      </c>
+      <c r="C19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" t="s">
         <v>109</v>
       </c>
-      <c r="B19" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" t="s">
-        <v>111</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="I19" t="s">
         <v>112</v>
-      </c>
-      <c r="I19" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" t="s">
+        <v>103</v>
+      </c>
+      <c r="I20" t="s">
         <v>105</v>
-      </c>
-      <c r="C20" t="s">
-        <v>106</v>
-      </c>
-      <c r="I20" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" t="s">
+        <v>119</v>
+      </c>
+      <c r="I22" t="s">
         <v>118</v>
-      </c>
-      <c r="C22" t="s">
-        <v>122</v>
-      </c>
-      <c r="I22" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" t="s">
         <v>124</v>
-      </c>
-      <c r="B23" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B25" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Worked my way up to All-Star Level 1; had Codex create an Agents file for deploying this pipeline
</commit_message>
<xml_diff>
--- a/Design/Workflow Sketch.xlsx
+++ b/Design/Workflow Sketch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llmdevice\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3997F65-22C6-4B65-8A40-E4B351816EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FA638B-5FB8-4F6D-9BFF-8F66BDB2C5A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="38580" windowHeight="21060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Have the workflow sketch reflect our change to package + demo organization
</commit_message>
<xml_diff>
--- a/Design/Workflow Sketch.xlsx
+++ b/Design/Workflow Sketch.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llmdevice\Design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llm-device\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FA638B-5FB8-4F6D-9BFF-8F66BDB2C5A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B469FAB-692B-404B-A2AD-12DEDC2F55F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="38580" windowHeight="21060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -231,9 +231,6 @@
     <t>Summary of driver installation</t>
   </si>
   <si>
-    <t>Make a physical device connection</t>
-  </si>
-  <si>
     <t>First, use Linux shell access to figure out this computer's details (e.g. ARMv7 with Debian 12.x.x).  Then, research necessary drivers and software that we would need for our device, without making decisions. We will ideally be doing this in Python on a a computer of this type. Don’t give step by step, just see if there will be necessary drivers. Report back if there are any major issues in the plan, like incompatibility. Only call out issues if it is specifically relevant to our plan and will cause potential major problems with our effort</t>
   </si>
   <si>
@@ -315,12 +312,6 @@
     <t>Design a step by step hello world per our plan, and explain your work. These steps will be followed by a domain expert scientist, not a software engineer, not a Linux sysadmin - so be clear. Agentically execute on this plan. Then, iterate on your mistakes and fix them until it all works.</t>
   </si>
   <si>
-    <t>Add more methods and settings into our Hello world script.</t>
-  </si>
-  <si>
-    <t>Add all planned-for methods and settings into our prior script.</t>
-  </si>
-  <si>
     <t>Write and debug a "hello, world" style demo script for our device</t>
   </si>
   <si>
@@ -430,6 +421,15 @@
   </si>
   <si>
     <t>Agentically assist the user through downloading and installing the necessary drivers for the device, so device is recognized on the computer. You also need any core, low-level Python libraries that would make basic hello, world type communication work.</t>
+  </si>
+  <si>
+    <t>Add more methods and settings into our Hello world script, and re-write it as a package that can be imported + a demo that can be run.</t>
+  </si>
+  <si>
+    <t>Make a physical device connection, with human help</t>
+  </si>
+  <si>
+    <t>Add all planned-for methods and settings into our prior MVP Level 1 package and demo.</t>
   </si>
 </sst>
 </file>
@@ -957,7 +957,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
         <v>49</v>
@@ -989,7 +989,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
@@ -1013,38 +1013,38 @@
         <v>14</v>
       </c>
       <c r="I8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
         <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>71</v>
       </c>
       <c r="H9" t="s">
         <v>14</v>
       </c>
       <c r="I9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -1053,7 +1053,7 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
@@ -1062,7 +1062,7 @@
         <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H10" t="s">
         <v>63</v>
@@ -1073,19 +1073,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H11" t="s">
         <v>63</v>
@@ -1096,13 +1096,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
         <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>133</v>
       </c>
       <c r="E12" t="s">
         <v>62</v>
@@ -1119,223 +1119,223 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C13" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
       <c r="F13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C14" t="s">
+        <v>132</v>
+      </c>
+      <c r="D14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
         <v>96</v>
       </c>
-      <c r="D14" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" t="s">
-        <v>99</v>
-      </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
         <v>97</v>
       </c>
-      <c r="D15" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" t="s">
-        <v>100</v>
-      </c>
       <c r="H15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B16" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" t="s">
         <v>110</v>
       </c>
-      <c r="B17" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" t="s">
-        <v>111</v>
-      </c>
-      <c r="E17" t="s">
-        <v>85</v>
-      </c>
-      <c r="F17" t="s">
-        <v>113</v>
-      </c>
       <c r="I17" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" t="s">
         <v>101</v>
-      </c>
-      <c r="E18" t="s">
-        <v>85</v>
-      </c>
-      <c r="F18" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" t="s">
         <v>106</v>
       </c>
-      <c r="B19" t="s">
-        <v>107</v>
-      </c>
-      <c r="C19" t="s">
-        <v>108</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="I19" t="s">
         <v>109</v>
-      </c>
-      <c r="I19" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" t="s">
+        <v>100</v>
+      </c>
+      <c r="I20" t="s">
         <v>102</v>
-      </c>
-      <c r="C20" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B21" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
+        <v>116</v>
+      </c>
+      <c r="I22" t="s">
         <v>115</v>
-      </c>
-      <c r="C22" t="s">
-        <v>119</v>
-      </c>
-      <c r="I22" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" t="s">
         <v>121</v>
-      </c>
-      <c r="B23" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Possibly no major changes; getting ready to modify the workflow
</commit_message>
<xml_diff>
--- a/Design/Workflow Sketch.xlsx
+++ b/Design/Workflow Sketch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llm-device\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B469FAB-692B-404B-A2AD-12DEDC2F55F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258E6864-FBCC-4991-935A-11B2F8C59C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -760,7 +760,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="56.6640625" customWidth="1"/>
     <col min="3" max="3" width="24.77734375" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>

</xml_diff>

<commit_message>
I noticed that my All-star and MVP Level 1 weren't creating libraries that looked like vendor libraries. I modified both instruction levels and combined them into Device Library Level 1, including requiring better documentation and a feel of vendor-provided software
</commit_message>
<xml_diff>
--- a/Design/Workflow Sketch.xlsx
+++ b/Design/Workflow Sketch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scott\Documents\SourceTree\llm-device\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258E6864-FBCC-4991-935A-11B2F8C59C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DA0868-9B46-4456-A6E3-F84C09850DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="28800" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="129">
   <si>
     <t>Stage</t>
   </si>
@@ -270,9 +270,6 @@
     <t>Hello Level 1</t>
   </si>
   <si>
-    <t>MVP Level 1</t>
-  </si>
-  <si>
     <t>Prototype - Level 1</t>
   </si>
   <si>
@@ -282,24 +279,6 @@
     <t>Documentation and examples of Facility control system</t>
   </si>
   <si>
-    <t>All-Star Level 1</t>
-  </si>
-  <si>
-    <t>Make a simulated version of this device in a way that talks with the facility control system. It has all the values and variables of All-Star Level 1 code, but none of the actual device. It exposes variables as if it were real, e.g. it has EPICS variables but does not actual device calls. Or, if not using EPICS, maybe it just makes up simulated numbers for volts/division instead of asking the device, etc.</t>
-  </si>
-  <si>
-    <t>Methods and Settings Plan, Hello Level 1</t>
-  </si>
-  <si>
-    <t>Methods and Settings Plan, MVP Level 1</t>
-  </si>
-  <si>
-    <t>MVP Level 1 Code</t>
-  </si>
-  <si>
-    <t>All-Star Level 1 Code</t>
-  </si>
-  <si>
     <t>Hello Level 1 Code</t>
   </si>
   <si>
@@ -315,21 +294,12 @@
     <t>Write and debug a "hello, world" style demo script for our device</t>
   </si>
   <si>
-    <t>Pick out a few key features to test from our list of methods and settings. Pick only the most important few for our main goals, that we could call an MVP implementation. Agentically execute on this plan. Then, iterate on your mistakes and fix them until it all works.</t>
-  </si>
-  <si>
-    <t>Start with our prior script, but now add all planned-for methods and settings into our prior script. Test as you go. Iterate on your mistakes and fix them until it all works.</t>
-  </si>
-  <si>
     <t>Make a simulated version of this device that speaks in the facility control system language.</t>
   </si>
   <si>
     <t>All-Star Level 2</t>
   </si>
   <si>
-    <t>Fill in the simulated version with the real calls, copying from All-Star Level 1.</t>
-  </si>
-  <si>
     <t>Simulated Level 2 Code</t>
   </si>
   <si>
@@ -405,9 +375,6 @@
     <t>Polishing - Level 1</t>
   </si>
   <si>
-    <t>HUMAN VETS ALL OF LEVEL 1 (importing All-star Level 1 as python library and running various commands)</t>
-  </si>
-  <si>
     <t>HUMAN VETS ALL OF LEVEL 2 (using the GUIs)</t>
   </si>
   <si>
@@ -423,13 +390,28 @@
     <t>Agentically assist the user through downloading and installing the necessary drivers for the device, so device is recognized on the computer. You also need any core, low-level Python libraries that would make basic hello, world type communication work.</t>
   </si>
   <si>
-    <t>Add more methods and settings into our Hello world script, and re-write it as a package that can be imported + a demo that can be run.</t>
-  </si>
-  <si>
     <t>Make a physical device connection, with human help</t>
   </si>
   <si>
-    <t>Add all planned-for methods and settings into our prior MVP Level 1 package and demo.</t>
+    <t>Device Library Level 1</t>
+  </si>
+  <si>
+    <t>If no manufacturer-provided Python library already exists, make a Python library wrapping all planned-for methods and settings.</t>
+  </si>
+  <si>
+    <t>Check if vendor already provided a library. Don't make a new library if one was already provided by the vendor. Test as you go. Iterate on your mistakes and fix them until it all works.</t>
+  </si>
+  <si>
+    <t>Device Library Code</t>
+  </si>
+  <si>
+    <t>HUMAN VETS ALL OF LEVEL 1 (importing Device Library 1 as python library and running various commands)</t>
+  </si>
+  <si>
+    <t>Fill in the simulated version with the real calls, copying from Device Library Level 1.</t>
+  </si>
+  <si>
+    <t>Make a simulated version of this device in a way that talks with the facility control system. It has all the values and variables of Level 1 code, but none of the actual device. It exposes variables as if it were real, e.g. it has EPICS variables but does not actual device calls. Or, if not using EPICS, maybe it just makes up simulated numbers for volts/division instead of asking the device, etc.</t>
   </si>
 </sst>
 </file>
@@ -756,20 +738,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="56.6640625" customWidth="1"/>
-    <col min="3" max="3" width="24.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="56.6328125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="8" width="49.44140625" customWidth="1"/>
-    <col min="9" max="9" width="28.33203125" customWidth="1"/>
-    <col min="10" max="10" width="30.77734375" customWidth="1"/>
+    <col min="6" max="8" width="49.453125" customWidth="1"/>
+    <col min="9" max="9" width="28.36328125" customWidth="1"/>
+    <col min="10" max="10" width="30.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -801,7 +783,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -830,7 +812,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -862,7 +844,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -894,7 +876,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -923,7 +905,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -955,9 +937,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
         <v>49</v>
@@ -987,9 +969,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
@@ -1016,9 +998,9 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
         <v>74</v>
@@ -1042,9 +1024,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
         <v>58</v>
@@ -1071,21 +1053,21 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="H11" t="s">
         <v>63</v>
@@ -1094,15 +1076,15 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
         <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="E12" t="s">
         <v>62</v>
@@ -1117,15 +1099,15 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
         <v>80</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D13" t="s">
         <v>76</v>
@@ -1137,205 +1119,176 @@
         <v>75</v>
       </c>
       <c r="G13" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="J13" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="C14" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D14" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E14" t="s">
         <v>8</v>
       </c>
       <c r="F14" t="s">
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="H14" t="s">
         <v>78</v>
       </c>
       <c r="I14" t="s">
+        <v>125</v>
+      </c>
+      <c r="J14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" t="s">
         <v>89</v>
       </c>
-      <c r="J14" t="s">
+      <c r="E17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C15" t="s">
-        <v>134</v>
-      </c>
-      <c r="D15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" t="s">
-        <v>97</v>
-      </c>
-      <c r="H15" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" t="s">
-        <v>90</v>
-      </c>
-      <c r="J15" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>125</v>
-      </c>
-      <c r="B16" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" t="s">
+        <v>106</v>
+      </c>
+      <c r="I21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" t="s">
         <v>107</v>
       </c>
-      <c r="B17" t="s">
-        <v>113</v>
-      </c>
-      <c r="C17" t="s">
-        <v>108</v>
-      </c>
-      <c r="E17" t="s">
-        <v>84</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="C22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
         <v>110</v>
       </c>
-      <c r="I17" t="s">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C18" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" t="s">
-        <v>105</v>
-      </c>
-      <c r="E19" t="s">
-        <v>106</v>
-      </c>
-      <c r="I19" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" t="s">
-        <v>99</v>
-      </c>
-      <c r="C20" t="s">
-        <v>100</v>
-      </c>
-      <c r="I20" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>123</v>
-      </c>
-      <c r="B21" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>111</v>
-      </c>
-      <c r="B22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" t="s">
-        <v>116</v>
-      </c>
-      <c r="I22" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>117</v>
-      </c>
-      <c r="C23" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>122</v>
-      </c>
-      <c r="B24" t="s">
-        <v>119</v>
-      </c>
-      <c r="C24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>124</v>
-      </c>
-      <c r="B25" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>